<commit_message>
Updated README, new transliteration of find and replace to make XML file of entire ms
</commit_message>
<xml_diff>
--- a/ReplaceIVTFFtoTEI.xlsx
+++ b/ReplaceIVTFFtoTEI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE40EB56-A17F-4FE0-980B-8BE0B1B472FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C1436-7255-40F5-8BC4-52476C2E84BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="912" windowWidth="7656" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
+    <workbookView xWindow="9528" yWindow="1128" windowWidth="7656" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="289">
   <si>
     <t>Voynich</t>
   </si>
@@ -902,6 +902,9 @@
   </si>
   <si>
     <t>the first twelve lines were written by Scribe 2, the rest Scribe 3</t>
+  </si>
+  <si>
+    <t>&lt;surface&gt;\n&lt;f\d\d?\d?r&gt;</t>
   </si>
 </sst>
 </file>
@@ -1544,6 +1547,9 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>288</v>
+      </c>
       <c r="D9" s="3" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
lots of changes and things. many such cases!
</commit_message>
<xml_diff>
--- a/ReplaceIVTFFtoTEI.xlsx
+++ b/ReplaceIVTFFtoTEI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C1436-7255-40F5-8BC4-52476C2E84BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F4276E-3D02-4EDB-A9CD-A6B0D4F46730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9528" yWindow="1128" windowWidth="7656" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
+    <workbookView xWindow="0" yWindow="288" windowWidth="11664" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="428">
   <si>
     <t>Voynich</t>
   </si>
@@ -560,49 +560,25 @@
     <t>@</t>
   </si>
   <si>
-    <t>Position of locus is unrelated to previous itemThe position of this locus is unrelated to the previous item, or not easily described by one of the following. This locator is always used for the first item on each page</t>
-  </si>
-  <si>
     <t>+</t>
   </si>
   <si>
-    <t>Generally below the previous item. This is the most common case</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
-    <t>At the start of the line below the previous item, but at the left margin, while the previous item was not.</t>
-  </si>
-  <si>
     <t>=</t>
   </si>
   <si>
-    <t>The locus is on the same line as the previous item but separated by some white space.</t>
-  </si>
-  <si>
     <t>&amp;</t>
   </si>
   <si>
-    <t>Similar to = but along a circular line</t>
-  </si>
-  <si>
     <t>~</t>
   </si>
   <si>
-    <t>Similar to = but the vertical alignment is not very good</t>
-  </si>
-  <si>
     <t>/</t>
   </si>
   <si>
-    <t>This locus is to the right of, and above the previous locus</t>
-  </si>
-  <si>
     <t>!</t>
-  </si>
-  <si>
-    <t>This locus refers to text that in reality does not exist in the MS.</t>
   </si>
   <si>
     <t>Locus Types</t>
@@ -905,6 +881,447 @@
   </si>
   <si>
     <t>&lt;surface&gt;\n&lt;f\d\d?\d?r&gt;</t>
+  </si>
+  <si>
+    <t>AT Position of locus is unrelated to previous item. The position of this locus is unrelated to the previous item, or not easily described by one of the following. This locator is always used for the first item on each page</t>
+  </si>
+  <si>
+    <t>AD Generally below the previous item. This is the most common case</t>
+  </si>
+  <si>
+    <t>AS At the start of the line below the previous item, but at the left margin, while the previous item was not.</t>
+  </si>
+  <si>
+    <t>AQ The locus is on the same line as the previous item but separated by some white space.</t>
+  </si>
+  <si>
+    <t>AN Similar to = but along a circular line</t>
+  </si>
+  <si>
+    <t>AM Similar to = but the vertical alignment is not very good</t>
+  </si>
+  <si>
+    <t>AL This locus is to the right of, and above the previous locus</t>
+  </si>
+  <si>
+    <t>AX This locus refers to text that in reality does not exist in the MS.</t>
+  </si>
+  <si>
+    <t>uva lupi</t>
+  </si>
+  <si>
+    <t>Plant IDs</t>
+  </si>
+  <si>
+    <t>aterpa belladonn[a]</t>
+  </si>
+  <si>
+    <t>solatrum d[iv|w]ale</t>
+  </si>
+  <si>
+    <t>solanum nigrum=morella</t>
+  </si>
+  <si>
+    <t>Cyanus segelis coeruleus (Kornblume)</t>
+  </si>
+  <si>
+    <t>centaurea (cf. Holm)</t>
+  </si>
+  <si>
+    <t>Collocasia</t>
+  </si>
+  <si>
+    <t>Egyptian lotus</t>
+  </si>
+  <si>
+    <t>Nymphoides Peltata (R. Zandbergen)</t>
+  </si>
+  <si>
+    <t>crassulatea (Cretan Dittany)</t>
+  </si>
+  <si>
+    <t>Hypericum</t>
+  </si>
+  <si>
+    <t>Centaurium Erythaea</t>
+  </si>
+  <si>
+    <t>Convulvula Ipomea? (climbing plant)</t>
+  </si>
+  <si>
+    <t>[Herba] Paris</t>
+  </si>
+  <si>
+    <t>Indian Cucumber?</t>
+  </si>
+  <si>
+    <t>Paretaria Urtica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asclepiades, but with wrong leaves (of Pediculum) </t>
+  </si>
+  <si>
+    <t>blackgum tree?</t>
+  </si>
+  <si>
+    <t>arctium?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidens(sp?)kyptis </t>
+  </si>
+  <si>
+    <t>polygonum persicaria</t>
+  </si>
+  <si>
+    <t>potentilla silvestris</t>
+  </si>
+  <si>
+    <t>oculus christi</t>
+  </si>
+  <si>
+    <t>Praenanthes</t>
+  </si>
+  <si>
+    <t>Atriplex hastata (spinach?)</t>
+  </si>
+  <si>
+    <t>Silene</t>
+  </si>
+  <si>
+    <t>Chelidonium Majus</t>
+  </si>
+  <si>
+    <t>Sallkraut</t>
+  </si>
+  <si>
+    <t>Herba Trinitatis</t>
+  </si>
+  <si>
+    <t>Freyschamkraut(sp?)</t>
+  </si>
+  <si>
+    <t>Scabiosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hellebore? </t>
+  </si>
+  <si>
+    <t>orientalis</t>
+  </si>
+  <si>
+    <t>Silene Aca[ul|nt]is</t>
+  </si>
+  <si>
+    <t>Leonotus or Leonarus</t>
+  </si>
+  <si>
+    <t>Tussilago petronitas</t>
+  </si>
+  <si>
+    <t>colto foot</t>
+  </si>
+  <si>
+    <t>Crassulatea Fetthenne</t>
+  </si>
+  <si>
+    <t>Pfeilkraut - scorpion</t>
+  </si>
+  <si>
+    <t>Sagittaria</t>
+  </si>
+  <si>
+    <t>Osmodei</t>
+  </si>
+  <si>
+    <t>Saw/Some thistle?</t>
+  </si>
+  <si>
+    <t>Herba Paris (liliacesus)</t>
+  </si>
+  <si>
+    <t>Herba Mortis</t>
+  </si>
+  <si>
+    <t>Canabis</t>
+  </si>
+  <si>
+    <t>Hemp</t>
+  </si>
+  <si>
+    <t>Ampfer(?)</t>
+  </si>
+  <si>
+    <t>Tamus communis</t>
+  </si>
+  <si>
+    <t>Polygonum dumetorum(sp?)</t>
+  </si>
+  <si>
+    <t>Smilax</t>
+  </si>
+  <si>
+    <t>trachaia leaves (Dioscorides fol/25r)</t>
+  </si>
+  <si>
+    <t>Moss Polytrichum</t>
+  </si>
+  <si>
+    <t>cranberry</t>
+  </si>
+  <si>
+    <t>mostly nettle- or mint-like</t>
+  </si>
+  <si>
+    <t>Leontopodium Edelweiss</t>
+  </si>
+  <si>
+    <t>unreadable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flower like artemisium absinth </t>
+  </si>
+  <si>
+    <t xml:space="preserve">wermuth but leaves are not </t>
+  </si>
+  <si>
+    <t>Verbena foenica</t>
+  </si>
+  <si>
+    <t>Asarium Europeum (Haselwurz)</t>
+  </si>
+  <si>
+    <t>Arum or Arisarum (Haselwurtz)</t>
+  </si>
+  <si>
+    <t>Holm) Dentaria(?) leaf only. Schippenwurtz?</t>
+  </si>
+  <si>
+    <t>Boragine</t>
+  </si>
+  <si>
+    <t>Hyrcio[unreadable] Arabum</t>
+  </si>
+  <si>
+    <t>Heracleum cervofilum</t>
+  </si>
+  <si>
+    <t>Mentastrum/Ros*(illegible)muentz</t>
+  </si>
+  <si>
+    <t>Campanula Ranunculus (Holm)</t>
+  </si>
+  <si>
+    <t>Archangelica</t>
+  </si>
+  <si>
+    <t>Glockenblume</t>
+  </si>
+  <si>
+    <t>Halskraut</t>
+  </si>
+  <si>
+    <t>Convolvulus erectus Same plant as f102r2[1,2]</t>
+  </si>
+  <si>
+    <t>smaller scabiosa</t>
+  </si>
+  <si>
+    <t>libanotus umbilifera</t>
+  </si>
+  <si>
+    <t>orchid root?</t>
+  </si>
+  <si>
+    <t>uva quercia (vitis)</t>
+  </si>
+  <si>
+    <t>oak/quercus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gall apple? </t>
+  </si>
+  <si>
+    <t>grape vine?</t>
+  </si>
+  <si>
+    <t>oak tree</t>
+  </si>
+  <si>
+    <t>Geranium</t>
+  </si>
+  <si>
+    <t>Indian hemp</t>
+  </si>
+  <si>
+    <t>Baldrian</t>
+  </si>
+  <si>
+    <t>Valerian</t>
+  </si>
+  <si>
+    <t>dwarf ceder(?)</t>
+  </si>
+  <si>
+    <t>illegible</t>
+  </si>
+  <si>
+    <t>Cickorium?</t>
+  </si>
+  <si>
+    <t>Lactuca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">crocus? </t>
+  </si>
+  <si>
+    <t>Primulaceon(?)</t>
+  </si>
+  <si>
+    <t>Primulaceon</t>
+  </si>
+  <si>
+    <t>Thistle</t>
+  </si>
+  <si>
+    <t>Gerneolem(?) Artichoke</t>
+  </si>
+  <si>
+    <t>Helianthus Tuberosus</t>
+  </si>
+  <si>
+    <t>Fern</t>
+  </si>
+  <si>
+    <t>Maidenhair fern???</t>
+  </si>
+  <si>
+    <t>Tansy?</t>
+  </si>
+  <si>
+    <t>Tropical Arum sagittarium visicating</t>
+  </si>
+  <si>
+    <t>crelpius(sp?) ranunculus</t>
+  </si>
+  <si>
+    <t>arum sagittarii</t>
+  </si>
+  <si>
+    <t>ranunculacea helleboria(?)</t>
+  </si>
+  <si>
+    <t>Antennaria Gnaphalium</t>
+  </si>
+  <si>
+    <t>Veratrum</t>
+  </si>
+  <si>
+    <t>Sentellaria</t>
+  </si>
+  <si>
+    <t>Veronica?</t>
+  </si>
+  <si>
+    <t>carnedris(sp)</t>
+  </si>
+  <si>
+    <t>Ehrenpreis?</t>
+  </si>
+  <si>
+    <t>Anchusa</t>
+  </si>
+  <si>
+    <t>Indian cucumber?</t>
+  </si>
+  <si>
+    <t>Toronicum Pardalianchus</t>
+  </si>
+  <si>
+    <t>Scamonia</t>
+  </si>
+  <si>
+    <t>Lunaria</t>
+  </si>
+  <si>
+    <t>Cyclamen</t>
+  </si>
+  <si>
+    <t>Artichoke</t>
+  </si>
+  <si>
+    <t>species of sunflower?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umbellifera? </t>
+  </si>
+  <si>
+    <t>Mandrake</t>
+  </si>
+  <si>
+    <t>Cow's tongue</t>
+  </si>
+  <si>
+    <t>Licopsis</t>
+  </si>
+  <si>
+    <t>Sedum Majus</t>
+  </si>
+  <si>
+    <t>Elecampane</t>
+  </si>
+  <si>
+    <t>leaves of boneset</t>
+  </si>
+  <si>
+    <t>Elephant's ear?</t>
+  </si>
+  <si>
+    <t>Boragine echium</t>
+  </si>
+  <si>
+    <t>Dianthus flower (convolvulus?)</t>
+  </si>
+  <si>
+    <t>Primula?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xerantrium? </t>
+  </si>
+  <si>
+    <t>Leaves of Osmuda regalis</t>
+  </si>
+  <si>
+    <t>Botriculum</t>
+  </si>
+  <si>
+    <t>Lunaria?</t>
+  </si>
+  <si>
+    <t>Mondform?</t>
+  </si>
+  <si>
+    <t>Banberry?</t>
+  </si>
+  <si>
+    <t>Actaea Waxberry</t>
+  </si>
+  <si>
+    <t>Wermut</t>
+  </si>
+  <si>
+    <t>Artemisium Absynthum</t>
+  </si>
+  <si>
+    <t>dipsaxus</t>
+  </si>
+  <si>
+    <t>calendula</t>
+  </si>
+  <si>
+    <t>Smilax tracheia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chenopodium </t>
   </si>
 </sst>
 </file>
@@ -1355,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D110CFE0-76A4-4947-8E53-2D23B2B7842A}">
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K209"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -1382,7 +1799,7 @@
         <v>45</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>172</v>
@@ -1405,7 +1822,7 @@
         <v>173</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>174</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1422,10 +1839,10 @@
         <v>7.5</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>176</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1448,10 +1865,10 @@
         <v>48</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>178</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1468,10 +1885,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>180</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -1494,10 +1911,10 @@
         <v>2</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>182</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1520,10 +1937,10 @@
         <v>3</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>184</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -1540,15 +1957,15 @@
         <v>4</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>186</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>10</v>
@@ -1563,10 +1980,10 @@
         <v>5</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>188</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1597,10 +2014,10 @@
         <v>7</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -1620,7 +2037,7 @@
         <v>93</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1637,10 +2054,10 @@
         <v>9</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -1657,10 +2074,10 @@
         <v>10</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1677,10 +2094,10 @@
         <v>11</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -1697,10 +2114,10 @@
         <v>12</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="4:11" x14ac:dyDescent="0.3">
@@ -1717,10 +2134,10 @@
         <v>13</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="4:11" x14ac:dyDescent="0.3">
@@ -1737,10 +2154,10 @@
         <v>14</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="4:11" x14ac:dyDescent="0.3">
@@ -1760,7 +2177,7 @@
         <v>92</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="4:11" x14ac:dyDescent="0.3">
@@ -1777,10 +2194,10 @@
         <v>17</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="4:11" x14ac:dyDescent="0.3">
@@ -1797,10 +2214,10 @@
         <v>19</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1817,10 +2234,10 @@
         <v>20</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1831,10 +2248,10 @@
         <v>187.5</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="4:11" x14ac:dyDescent="0.3">
@@ -1851,10 +2268,10 @@
         <v>94</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="4:11" x14ac:dyDescent="0.3">
@@ -1871,10 +2288,10 @@
         <v>1</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="4:11" x14ac:dyDescent="0.3">
@@ -1891,10 +2308,10 @@
         <v>2</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="4:11" x14ac:dyDescent="0.3">
@@ -1911,10 +2328,10 @@
         <v>3</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" spans="4:11" x14ac:dyDescent="0.3">
@@ -1931,10 +2348,10 @@
         <v>4</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="4:11" x14ac:dyDescent="0.3">
@@ -1951,10 +2368,10 @@
         <v>5</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="4:11" x14ac:dyDescent="0.3">
@@ -1974,7 +2391,7 @@
         <v>91</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="4:11" x14ac:dyDescent="0.3">
@@ -1991,10 +2408,10 @@
         <v>7</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="4:11" x14ac:dyDescent="0.3">
@@ -2011,10 +2428,10 @@
         <v>8</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="4:11" x14ac:dyDescent="0.3">
@@ -2031,10 +2448,10 @@
         <v>9</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="4:11" x14ac:dyDescent="0.3">
@@ -2051,10 +2468,10 @@
         <v>10</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2071,10 +2488,10 @@
         <v>11</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
     <row r="36" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2105,7 +2522,7 @@
         <v>13</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="K37" s="2"/>
     </row>
@@ -2123,10 +2540,10 @@
         <v>14</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="4:11" x14ac:dyDescent="0.3">
@@ -2143,10 +2560,10 @@
         <v>15</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2163,10 +2580,10 @@
         <v>16</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="4:11" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2177,10 +2594,10 @@
         <v>17</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.3">
@@ -2194,7 +2611,7 @@
         <v>24</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43" spans="4:11" x14ac:dyDescent="0.3">
@@ -2208,7 +2625,7 @@
         <v>173</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" spans="4:11" x14ac:dyDescent="0.3">
@@ -2219,10 +2636,10 @@
         <v>20</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="4:11" x14ac:dyDescent="0.3">
@@ -2233,10 +2650,10 @@
         <v>21</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" spans="4:11" x14ac:dyDescent="0.3">
@@ -2247,10 +2664,10 @@
         <v>22</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
     </row>
     <row r="47" spans="4:11" x14ac:dyDescent="0.3">
@@ -2261,10 +2678,10 @@
         <v>23</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="48" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2275,18 +2692,18 @@
         <v>24</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
     </row>
     <row r="49" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="J49" s="8" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="50" spans="7:11" x14ac:dyDescent="0.3">
@@ -2297,10 +2714,10 @@
         <v>103</v>
       </c>
       <c r="J50" s="8" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="51" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2309,10 +2726,10 @@
       </c>
       <c r="H51" s="4"/>
       <c r="J51" s="7" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2327,7 +2744,7 @@
       </c>
       <c r="H53" s="4"/>
       <c r="J53" s="1" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="K53" s="2"/>
     </row>
@@ -2337,10 +2754,10 @@
       </c>
       <c r="H54" s="4"/>
       <c r="J54" s="8" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="55" spans="7:11" x14ac:dyDescent="0.3">
@@ -2352,7 +2769,7 @@
         <v>173</v>
       </c>
       <c r="K55" s="4" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="56" spans="7:11" x14ac:dyDescent="0.3">
@@ -2361,10 +2778,10 @@
       </c>
       <c r="H56" s="4"/>
       <c r="J56" s="8" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="57" spans="7:11" ht="43.2" x14ac:dyDescent="0.3">
@@ -2373,10 +2790,10 @@
       </c>
       <c r="H57" s="4"/>
       <c r="J57" s="8" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="K57" s="9" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="58" spans="7:11" x14ac:dyDescent="0.3">
@@ -2385,10 +2802,10 @@
       </c>
       <c r="H58" s="4"/>
       <c r="J58" s="8" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
     </row>
     <row r="59" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2397,10 +2814,10 @@
       </c>
       <c r="H59" s="4"/>
       <c r="J59" s="7" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
     </row>
     <row r="60" spans="7:11" x14ac:dyDescent="0.3">
@@ -2409,10 +2826,10 @@
       </c>
       <c r="H60" s="4"/>
       <c r="J60" s="8" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="K60" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
     </row>
     <row r="61" spans="7:11" x14ac:dyDescent="0.3">
@@ -2421,10 +2838,10 @@
       </c>
       <c r="H61" s="4"/>
       <c r="J61" s="8" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="K61" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
     </row>
     <row r="62" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2435,10 +2852,10 @@
     </row>
     <row r="63" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="J63" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="K63" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="64" spans="7:11" x14ac:dyDescent="0.3">
@@ -2449,305 +2866,947 @@
         <v>117</v>
       </c>
     </row>
-    <row r="65" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G65" s="8" t="s">
         <v>118</v>
       </c>
       <c r="H65" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K65" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="66" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G66" s="8" t="s">
         <v>119</v>
       </c>
       <c r="H66" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="67" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K66" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="67" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G67" s="8" t="s">
         <v>120</v>
       </c>
       <c r="H67" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="68" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K67" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="68" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G68" s="8" t="s">
         <v>121</v>
       </c>
       <c r="H68" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="69" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K68" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="69" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G69" s="8" t="s">
         <v>122</v>
       </c>
       <c r="H69" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="70" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K69" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="70" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G70" s="7" t="s">
         <v>123</v>
       </c>
       <c r="H70" s="6">
         <v>6</v>
       </c>
-    </row>
-    <row r="71" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="72" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K70" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="71" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K71" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="72" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G72" s="1" t="s">
         <v>124</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="73" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K72" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="73" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G73" s="8" t="s">
         <v>134</v>
       </c>
       <c r="H73" s="4" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="74" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K73" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="74" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G74" s="8" t="s">
         <v>135</v>
       </c>
       <c r="H74" s="4" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="75" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K74" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="75" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G75" s="8" t="s">
         <v>136</v>
       </c>
       <c r="H75" s="4" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="76" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K75" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="76" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G76" s="8" t="s">
         <v>137</v>
       </c>
       <c r="H76" s="4" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="77" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K76" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="77" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G77" s="8" t="s">
         <v>138</v>
       </c>
       <c r="H77" s="4" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="78" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K77" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="78" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G78" s="8" t="s">
         <v>140</v>
       </c>
       <c r="H78" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="79" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K78" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="79" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G79" s="8" t="s">
         <v>139</v>
       </c>
       <c r="H79" s="4" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="80" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K79" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="80" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G80" s="7" t="s">
         <v>141</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="81" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="82" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K80" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="81" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K81" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="82" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G82" s="1" t="s">
         <v>142</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="83" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K82" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="83" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G83" s="8" t="s">
         <v>144</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="84" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+      <c r="K83" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="84" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G84" s="7" t="s">
         <v>145</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="85" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="86" spans="7:8" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+      <c r="K84" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="85" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K85" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="86" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G86" s="1" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="87" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K86" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="87" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G87" s="8" t="s">
         <v>146</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="88" spans="7:8" x14ac:dyDescent="0.3">
+        <v>271</v>
+      </c>
+      <c r="K87" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="88" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G88" s="8" t="s">
         <v>147</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="89" spans="7:8" x14ac:dyDescent="0.3">
+        <v>272</v>
+      </c>
+      <c r="K88" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="89" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G89" s="8" t="s">
         <v>148</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="90" spans="7:8" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+      <c r="K89" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="90" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G90" s="8" t="s">
         <v>149</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="91" spans="7:8" x14ac:dyDescent="0.3">
+        <v>274</v>
+      </c>
+      <c r="K90" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="91" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G91" s="8" t="s">
         <v>150</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="92" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+      <c r="K91" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="92" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G92" s="7" t="s">
         <v>151</v>
       </c>
       <c r="H92" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="93" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="94" spans="7:8" x14ac:dyDescent="0.3">
+        <v>279</v>
+      </c>
+      <c r="K92" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="93" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K93" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="94" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G94" s="1" t="s">
         <v>153</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="95" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K94" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="95" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G95" s="8" t="s">
         <v>154</v>
       </c>
       <c r="H95" s="4"/>
-    </row>
-    <row r="96" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K95" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="96" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G96" s="8" t="s">
         <v>155</v>
       </c>
       <c r="H96" s="4"/>
-    </row>
-    <row r="97" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K96" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="97" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G97" s="8" t="s">
         <v>156</v>
       </c>
       <c r="H97" s="4"/>
-    </row>
-    <row r="98" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K97" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="98" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G98" s="8" t="s">
         <v>157</v>
       </c>
       <c r="H98" s="4"/>
-    </row>
-    <row r="99" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K98" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="99" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G99" s="8" t="s">
         <v>158</v>
       </c>
       <c r="H99" s="4"/>
-    </row>
-    <row r="100" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K99" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="100" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G100" s="8" t="s">
         <v>159</v>
       </c>
       <c r="H100" s="4"/>
-    </row>
-    <row r="101" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K100" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="101" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G101" s="7" t="s">
         <v>160</v>
       </c>
       <c r="H101" s="6"/>
-    </row>
-    <row r="102" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="103" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K101" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="102" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K102" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="103" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G103" s="1" t="s">
         <v>161</v>
       </c>
       <c r="H103" s="2"/>
-    </row>
-    <row r="104" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K103" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="104" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G104" s="8" t="s">
         <v>162</v>
       </c>
       <c r="H104" s="4" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="105" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K104" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="105" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G105" s="8" t="s">
         <v>163</v>
       </c>
       <c r="H105" s="4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="106" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K105" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="106" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G106" s="8" t="s">
         <v>164</v>
       </c>
       <c r="H106" s="4" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="107" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="K106" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="107" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G107" s="8" t="s">
         <v>165</v>
       </c>
       <c r="H107" s="4" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="108" spans="7:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K107" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="108" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G108" s="7" t="s">
         <v>166</v>
       </c>
       <c r="H108" s="6" t="s">
         <v>171</v>
+      </c>
+      <c r="K108" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="109" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="K109" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="110" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="K110" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="111" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="K111" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="112" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="K112" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="113" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K113" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="114" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K114" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="115" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K115" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="116" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K116" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="117" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K117" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="118" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K118" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="119" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K119" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="120" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K120" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="121" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K121" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="122" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K122" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="123" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K123" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="124" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K124" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="125" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K125" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="126" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K126" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="127" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K127" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="128" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K128" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="129" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K129" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="130" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K130" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="131" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K131" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="132" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K132" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="133" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K133" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="134" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K134" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="135" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K135" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="136" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K136" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="137" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K137" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="138" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K138" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="139" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K139" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="140" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K140" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="141" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K141" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="142" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K142" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="143" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K143" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="144" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K144" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="145" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K145" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="146" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K146" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="147" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K147" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="148" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K148" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="149" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K149" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="150" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K150" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="151" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K151" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="152" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K152" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="153" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K153" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="154" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K154" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="155" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K155" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="156" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K156" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="157" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K157" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="158" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K158" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="159" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K159" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="160" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K160" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="161" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K161" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="162" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K162" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="163" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K163" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="164" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K164" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="165" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K165" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="166" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K166" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="167" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K167" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="168" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K168" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="169" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K169" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="170" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K170" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="171" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K171" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="172" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K172" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="173" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K173" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="174" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K174" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="175" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K175" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="176" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K176" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="177" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K177" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="178" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K178" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="179" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K179" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="180" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K180" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="181" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K181" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="182" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K182" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="183" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K183" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="184" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K184" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="185" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K185" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="186" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K186" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="187" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K187" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="188" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K188" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="189" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K189" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="190" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K190" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="191" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K191" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="192" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K192" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="193" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K193" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="194" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K194" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="195" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K195" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="196" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K196" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="197" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K197" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="198" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K198" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="199" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K199" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="200" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K200" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="201" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K201" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="202" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K202" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="203" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K203" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="204" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K204" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="205" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K205" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="206" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K206" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="207" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K207" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="208" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K208" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="209" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K209" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
creating a new python file for future transliteration files
</commit_message>
<xml_diff>
--- a/ReplaceIVTFFtoTEI.xlsx
+++ b/ReplaceIVTFFtoTEI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F4276E-3D02-4EDB-A9CD-A6B0D4F46730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60D8347-5E46-4719-B933-22226193E32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="288" windowWidth="11664" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -335,12 +335,6 @@
     <t>End of Paragraph</t>
   </si>
   <si>
-    <t>&lt;p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>&lt;\$&gt;</t>
   </si>
   <si>
@@ -1322,6 +1316,12 @@
   </si>
   <si>
     <t xml:space="preserve">Chenopodium </t>
+  </si>
+  <si>
+    <t>&lt;zone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;/zone&gt;</t>
   </si>
 </sst>
 </file>
@@ -1799,10 +1799,10 @@
         <v>45</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1819,10 +1819,10 @@
         <v>46</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1839,10 +1839,10 @@
         <v>7.5</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1850,7 +1850,7 @@
         <v>96</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>99</v>
+        <v>426</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>5</v>
@@ -1865,10 +1865,10 @@
         <v>48</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1885,10 +1885,10 @@
         <v>1</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -1911,18 +1911,18 @@
         <v>2</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>100</v>
+        <v>427</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>8</v>
@@ -1937,10 +1937,10 @@
         <v>3</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -1957,15 +1957,15 @@
         <v>4</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>10</v>
@@ -1980,10 +1980,10 @@
         <v>5</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2014,10 +2014,10 @@
         <v>7</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -2037,7 +2037,7 @@
         <v>93</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -2054,10 +2054,10 @@
         <v>9</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -2074,10 +2074,10 @@
         <v>10</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -2094,10 +2094,10 @@
         <v>11</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -2114,10 +2114,10 @@
         <v>12</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" spans="4:11" x14ac:dyDescent="0.3">
@@ -2134,10 +2134,10 @@
         <v>13</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="4:11" x14ac:dyDescent="0.3">
@@ -2154,10 +2154,10 @@
         <v>14</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="4:11" x14ac:dyDescent="0.3">
@@ -2177,7 +2177,7 @@
         <v>92</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="4:11" x14ac:dyDescent="0.3">
@@ -2194,10 +2194,10 @@
         <v>17</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="4:11" x14ac:dyDescent="0.3">
@@ -2214,10 +2214,10 @@
         <v>19</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2234,10 +2234,10 @@
         <v>20</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2248,10 +2248,10 @@
         <v>187.5</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="24" spans="4:11" x14ac:dyDescent="0.3">
@@ -2268,10 +2268,10 @@
         <v>94</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25" spans="4:11" x14ac:dyDescent="0.3">
@@ -2288,10 +2288,10 @@
         <v>1</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26" spans="4:11" x14ac:dyDescent="0.3">
@@ -2308,10 +2308,10 @@
         <v>2</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="4:11" x14ac:dyDescent="0.3">
@@ -2328,10 +2328,10 @@
         <v>3</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" spans="4:11" x14ac:dyDescent="0.3">
@@ -2348,10 +2348,10 @@
         <v>4</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="29" spans="4:11" x14ac:dyDescent="0.3">
@@ -2368,10 +2368,10 @@
         <v>5</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="30" spans="4:11" x14ac:dyDescent="0.3">
@@ -2391,7 +2391,7 @@
         <v>91</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="4:11" x14ac:dyDescent="0.3">
@@ -2408,10 +2408,10 @@
         <v>7</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" spans="4:11" x14ac:dyDescent="0.3">
@@ -2428,10 +2428,10 @@
         <v>8</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="33" spans="4:11" x14ac:dyDescent="0.3">
@@ -2448,10 +2448,10 @@
         <v>9</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="34" spans="4:11" x14ac:dyDescent="0.3">
@@ -2468,10 +2468,10 @@
         <v>10</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2488,10 +2488,10 @@
         <v>11</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="36" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2522,7 +2522,7 @@
         <v>13</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="K37" s="2"/>
     </row>
@@ -2540,10 +2540,10 @@
         <v>14</v>
       </c>
       <c r="J38" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="39" spans="4:11" x14ac:dyDescent="0.3">
@@ -2560,10 +2560,10 @@
         <v>15</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="40" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2580,10 +2580,10 @@
         <v>16</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="41" spans="4:11" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2594,10 +2594,10 @@
         <v>17</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="4:11" x14ac:dyDescent="0.3">
@@ -2611,7 +2611,7 @@
         <v>24</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="43" spans="4:11" x14ac:dyDescent="0.3">
@@ -2622,10 +2622,10 @@
         <v>19</v>
       </c>
       <c r="J43" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="44" spans="4:11" x14ac:dyDescent="0.3">
@@ -2636,10 +2636,10 @@
         <v>20</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="45" spans="4:11" x14ac:dyDescent="0.3">
@@ -2650,10 +2650,10 @@
         <v>21</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="46" spans="4:11" x14ac:dyDescent="0.3">
@@ -2664,10 +2664,10 @@
         <v>22</v>
       </c>
       <c r="J46" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="47" spans="4:11" x14ac:dyDescent="0.3">
@@ -2678,10 +2678,10 @@
         <v>23</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="48" spans="4:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2692,1121 +2692,1121 @@
         <v>24</v>
       </c>
       <c r="J48" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="J49" s="8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="50" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G50" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J50" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="51" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G51" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H51" s="4"/>
       <c r="J51" s="7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="52" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G52" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H52" s="4"/>
     </row>
     <row r="53" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G53" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H53" s="4"/>
       <c r="J53" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="K53" s="2"/>
     </row>
     <row r="54" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G54" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H54" s="4"/>
       <c r="J54" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="55" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G55" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H55" s="4"/>
       <c r="J55" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K55" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="56" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G56" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H56" s="4"/>
       <c r="J56" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="57" spans="7:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="G57" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H57" s="4"/>
       <c r="J57" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="K57" s="9" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="58" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G58" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H58" s="4"/>
       <c r="J58" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G59" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H59" s="4"/>
       <c r="J59" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G60" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H60" s="4"/>
       <c r="J60" s="8" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="K60" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="61" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G61" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H61" s="4"/>
       <c r="J61" s="8" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="K61" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="62" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G62" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H62" s="6"/>
     </row>
     <row r="63" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="J63" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K63" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="64" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G64" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="65" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G65" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H65" s="4">
         <v>1</v>
       </c>
       <c r="K65" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="66" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G66" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H66" s="4">
         <v>2</v>
       </c>
       <c r="K66" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="67" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G67" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H67" s="4">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="68" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G68" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H68" s="4">
         <v>4</v>
       </c>
       <c r="K68" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="69" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G69" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H69" s="4">
         <v>5</v>
       </c>
       <c r="K69" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="70" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G70" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H70" s="6">
         <v>6</v>
       </c>
       <c r="K70" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="71" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="K71" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="72" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G72" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K72" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="73" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G73" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K73" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="74" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G74" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K74" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="75" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G75" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K75" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="76" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G76" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K76" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="77" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G77" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K77" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="78" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G78" s="8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K78" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="79" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G79" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K79" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="80" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G80" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K80" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="81" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="K81" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="82" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G82" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="K82" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="83" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G83" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K83" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="84" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G84" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="K84" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="85" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="K85" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="86" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G86" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K86" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="87" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G87" s="8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="K87" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="88" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G88" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="K88" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="89" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G89" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="K89" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="90" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G90" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="K90" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="91" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G91" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="K91" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="92" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G92" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H92" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="K92" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="93" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="K93" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="94" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G94" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K94" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="95" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G95" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H95" s="4"/>
       <c r="K95" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="96" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G96" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H96" s="4"/>
       <c r="K96" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="97" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G97" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H97" s="4"/>
       <c r="K97" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="98" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G98" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H98" s="4"/>
       <c r="K98" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="99" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G99" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H99" s="4"/>
       <c r="K99" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="100" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G100" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H100" s="4"/>
       <c r="K100" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="101" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G101" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H101" s="6"/>
       <c r="K101" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="102" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="K102" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="103" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G103" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H103" s="2"/>
       <c r="K103" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="104" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G104" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H104" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K104" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="105" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G105" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H105" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K105" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="106" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G106" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H106" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K106" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="107" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G107" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H107" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K107" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="108" spans="7:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G108" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K108" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="109" spans="7:11" x14ac:dyDescent="0.3">
       <c r="K109" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="110" spans="7:11" x14ac:dyDescent="0.3">
       <c r="K110" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="111" spans="7:11" x14ac:dyDescent="0.3">
       <c r="K111" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="112" spans="7:11" x14ac:dyDescent="0.3">
       <c r="K112" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="113" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K113" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="114" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K114" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="115" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K115" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="116" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K116" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="117" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K117" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="118" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K118" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="119" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K119" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="120" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K120" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="121" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K121" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="122" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K122" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="123" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K123" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="124" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K124" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="125" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K125" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="126" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K126" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="127" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K127" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="128" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K128" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="129" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K129" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="130" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K130" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="131" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K131" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="132" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K132" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="133" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K133" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="134" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K134" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="135" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K135" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="136" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K136" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="137" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K137" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="138" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K138" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="139" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K139" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="140" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K140" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="141" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K141" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="142" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K142" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="143" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K143" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="144" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K144" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="145" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K145" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="146" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K146" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="147" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K147" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="148" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K148" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="149" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K149" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="150" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K150" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="151" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K151" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="152" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K152" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="153" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K153" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="154" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K154" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="155" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K155" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="156" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K156" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="157" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K157" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="158" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K158" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="159" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K159" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="160" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K160" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="161" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K161" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="162" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K162" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="163" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K163" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="164" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K164" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="165" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K165" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="166" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K166" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="167" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K167" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="168" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K168" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="169" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K169" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="170" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K170" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="171" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K171" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="172" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K172" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="173" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K173" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="174" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K174" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="175" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K175" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="176" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K176" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="177" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K177" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="178" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K178" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="179" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K179" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="180" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K180" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="181" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K181" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="182" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K182" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="183" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K183" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="184" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K184" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="185" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K185" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="186" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K186" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="187" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K187" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="188" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K188" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="189" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K189" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="190" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K190" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="191" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K191" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="192" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K192" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="193" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K193" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="194" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K194" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="195" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K195" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="196" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K196" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="197" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K197" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="198" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K198" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="199" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K199" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="200" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K200" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="201" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K201" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="202" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K202" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="203" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K203" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="204" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K204" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="205" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K205" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="206" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K206" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="207" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K207" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="208" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K208" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="209" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K209" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>